<commit_message>
Consolidate management specification with Co-Owner and P0 P1 contracts
</commit_message>
<xml_diff>
--- a/docs/02-requirements/requirements-traceability-matrix.xlsx
+++ b/docs/02-requirements/requirements-traceability-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Requirements traceability'!$A$1:$F$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Requirements traceability'!$A$1:$F$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -62,10 +62,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -145,7 +148,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RequirementsTraceability" displayName="RequirementsTraceability" ref="A1:F21" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RequirementsTraceability" displayName="RequirementsTraceability" ref="A1:F33" headerRowCount="1">
   <autoFilter ref="A1:F21"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Requirement ID"/>
@@ -448,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -514,12 +517,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Automated T1/T2 passed</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Real-session expiry remains untested</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
         </is>
       </c>
     </row>
@@ -546,12 +549,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Implemented / not integration-tested</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Public key and real QA account needed</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
         </is>
       </c>
     </row>
@@ -578,12 +581,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Demo/config-error case passed; real flow not run</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Confirmation policy/project setup pending</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
         </is>
       </c>
     </row>
@@ -610,12 +613,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Unconfigured case passed; real flow not run</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Mailbox/provider access needed</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
         </is>
       </c>
     </row>
@@ -642,12 +645,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Implemented / not integration-tested</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Recovery variants and invalid links not run</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
         </is>
       </c>
     </row>
@@ -674,12 +677,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Demo case passed</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Business UAT pending</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
         </is>
       </c>
     </row>
@@ -706,12 +709,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Demo persistence passed; server save not run</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Real metadata update needed</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
         </is>
       </c>
     </row>
@@ -738,12 +741,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Demo controls passed; real reset not run</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Native install not run</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
         </is>
       </c>
     </row>
@@ -770,12 +773,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Demo logout passed; real logout not run</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Session invalidation review pending</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
         </is>
       </c>
     </row>
@@ -787,27 +790,27 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Explicit separated demo</t>
+          <t>Retired historical demo requirement; no demo access permitted</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>App enterDemo/sessionStorage</t>
+          <t>src/main.jsx sample cleanup; session-only gate</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>TC-02, TC-04, TC-08</t>
+          <t>tests/unconfigured.spec.js</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Automated demo cases passed</t>
+          <t>Retired; not current product scope</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Demo is not a backend identity</t>
+          <t>Never recycle this requirement ID or restore demo mode</t>
         </is>
       </c>
     </row>
@@ -834,12 +837,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>390/320px Chromium passed</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Other devices/browser matrix pending</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
         </is>
       </c>
     </row>
@@ -866,12 +869,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Instructions/offline shell passed</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Native install/upgrade pending</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
         </is>
       </c>
     </row>
@@ -898,12 +901,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Partially tested</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>768/1440 matrix to approve</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
         </is>
       </c>
     </row>
@@ -930,12 +933,12 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Not audited</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>AA conformance not established</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
         </is>
       </c>
     </row>
@@ -962,12 +965,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Dependency audit only</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Security/headers/real auth pending</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
         </is>
       </c>
     </row>
@@ -994,12 +997,12 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Passed locally</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>CI absent</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
         </is>
       </c>
     </row>
@@ -1026,12 +1029,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Login shell passed</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Upgrade/mutation failure paths pending</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
         </is>
       </c>
     </row>
@@ -1058,12 +1061,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Not measured</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>No benchmark acceptance</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
         </is>
       </c>
     </row>
@@ -1090,12 +1093,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Not defined or tested</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>RTO/RPO/SLA and owners TBD</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
         </is>
       </c>
     </row>
@@ -1122,17 +1125,401 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Chromium only</t>
+          <t>Current requirement/coverage mapping; not rerun for documentation update</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Safari/Firefox/Edge/real devices pending</t>
+          <t>See refreshed SRS/current code; old demo/setup evidence is historical. Real-provider/independent review remains pending as applicable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="58" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>MGT-01</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Organization operators vs branch staff isolation</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Planned: docs/11-management-plan/README.md</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>GOV-01, GOV-02, GOV-05; DBF-03/04</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Specified; not implemented / not executed</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Phase entry approvals and executed evidence required; no management code deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="58" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>MGT-02</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Operational Co-Owner with Owner-only ownership/security</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Planned: docs/11-management-plan/README.md</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>GOV-03, GOV-04</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Specified; not implemented / not executed</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Phase entry approvals and executed evidence required; no management code deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="58" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>MGT-03</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Phase 1 idempotency, audit atomicity and external recovery</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Planned: docs/11-management-plan/README.md</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>GOV-06–GOV-09; DBF-08/11</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Specified; not implemented / not executed</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Phase entry approvals and executed evidence required; no management code deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="58" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>MGT-04</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Typed per-phase supporting schema/least privilege</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Planned: docs/11-management-plan/README.md</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>GOV-10; DBF-02/04</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Specified; not implemented / not executed</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Phase entry approvals and executed evidence required; no management code deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="58" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>MGT-05</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Instructor-observed auto-class attendance, no student writes</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Planned: docs/11-management-plan/README.md</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>ATT-01–ATT-17</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Specified; not implemented / not executed</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Phase entry approvals and executed evidence required; no management code deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="58" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>MGT-06</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Independent bounded Admin attendance capabilities</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Planned: docs/11-management-plan/README.md</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>GOV-11–GOV-14; ATT-10</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Specified; not implemented / not executed</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Phase entry approvals and executed evidence required; no management code deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="58" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>MGT-07</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Both monthly policies and immutable exact-money billing</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Planned: docs/11-management-plan/README.md</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>BIL-01–BIL-16; GOV-15</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Specified; not implemented / not executed</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Phase entry approvals and executed evidence required; no management code deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="58" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>MGT-08</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Audited manual payments/refunds and safe statements</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Planned: docs/11-management-plan/README.md</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>BIL-09–BIL-16; DBF-08</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Specified; not implemented / not executed</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Phase entry approvals and executed evidence required; no management code deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="58" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>MGT-09</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>RPC-only bounded reads/writes and measured workload</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Planned: docs/11-management-plan/README.md</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>DBF-01–DBF-12; GOV-15</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Specified; not implemented / not executed</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Phase entry approvals and executed evidence required; no management code deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="58" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>MGT-10</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Existing-user/profile migration and failure reconciliation</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Planned: docs/11-management-plan/README.md</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>GOV-08/09/16</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Specified; not implemented / not executed</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Phase entry approvals and executed evidence required; no management code deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="58" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>MGT-11</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Privacy/retention/restore/operational accountability</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Planned: docs/11-management-plan/README.md</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>GOV-16; production decision register</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Specified; not implemented / not executed</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Phase entry approvals and executed evidence required; no management code deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="58" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>MGT-12</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Phase entry/exit evidence, five-role UAT and approvals</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Planned: docs/11-management-plan/README.md</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Consolidated phase-readiness matrix</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Specified; not implemented / not executed</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Phase entry approvals and executed evidence required; no management code deployed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F21"/>
+  <autoFilter ref="A1:F33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1146,7 +1533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1173,7 +1560,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Draft; approvals pending</t>
+          <t>Draft approvals pending; 20 stable app IDs (FR-10 retired) plus 12 specified management requirements</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1572,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>92f42e3</t>
+          <t>Current application 1.1.1 / f72bee4; consolidated management plan 0.4</t>
         </is>
       </c>
     </row>
@@ -1210,6 +1597,18 @@
       <c r="B5" t="inlineStr">
         <is>
           <t>Verification is case-specific; implementation does not imply tested or accepted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Evidence boundary</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Coverage mappings are not a new test run. Management implementation/live evidence and formal approvals pending.</t>
         </is>
       </c>
     </row>

</xml_diff>